<commit_message>
updated data analysis notebooks and example data
</commit_message>
<xml_diff>
--- a/content/computational_sets/data_analysis_example_data_sets.xlsx
+++ b/content/computational_sets/data_analysis_example_data_sets.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10726"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\Pchem\3141 Lab\Fall 2026\Activities\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jfoley19/Code/chem3141-book/content/computational_sets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7F654280-EB19-45CE-8E75-D3D0E339D536}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BD9551F-4CB7-4A41-AFCE-9F814D4A3ADE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{E33697AF-AC8F-4076-A4E0-31882C04577A}"/>
+    <workbookView xWindow="22980" yWindow="2100" windowWidth="43560" windowHeight="17780" activeTab="5" xr2:uid="{E33697AF-AC8F-4076-A4E0-31882C04577A}"/>
   </bookViews>
   <sheets>
     <sheet name="Exercise A Data" sheetId="1" r:id="rId1"/>
@@ -19,6 +19,7 @@
     <sheet name="Exercise B Dataset 2" sheetId="4" r:id="rId4"/>
     <sheet name="Exercise C Data" sheetId="5" r:id="rId5"/>
     <sheet name="Exercise C Dataset 2" sheetId="6" r:id="rId6"/>
+    <sheet name="Sheet1" sheetId="7" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -298,9 +299,6 @@
     <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -309,6 +307,9 @@
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -645,14 +646,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BFDAC1E3-44A8-4C9E-A53C-7D577177392E}">
   <dimension ref="A1:G25"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -673,7 +674,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" s="3">
         <v>26.4</v>
       </c>
@@ -694,7 +695,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" s="3">
         <v>25.2</v>
       </c>
@@ -706,7 +707,7 @@
       </c>
       <c r="D3" s="2"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" s="3">
         <v>24.1</v>
       </c>
@@ -718,7 +719,7 @@
       </c>
       <c r="D4" s="2"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" s="3">
         <v>23.2</v>
       </c>
@@ -730,7 +731,7 @@
       </c>
       <c r="D5" s="2"/>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" s="3">
         <v>22.1</v>
       </c>
@@ -742,7 +743,7 @@
       </c>
       <c r="D6" s="2"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" s="3">
         <v>20.7</v>
       </c>
@@ -754,7 +755,7 @@
       </c>
       <c r="D7" s="2"/>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" s="3">
         <v>19.600000000000001</v>
       </c>
@@ -766,7 +767,7 @@
       </c>
       <c r="D8" s="2"/>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" s="3">
         <v>18.5</v>
       </c>
@@ -778,7 +779,7 @@
       </c>
       <c r="D9" s="2"/>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" s="3">
         <v>17.2</v>
       </c>
@@ -790,7 +791,7 @@
       </c>
       <c r="D10" s="2"/>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" s="3">
         <v>16.100000000000001</v>
       </c>
@@ -802,7 +803,7 @@
       </c>
       <c r="D11" s="2"/>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" s="3">
         <v>14.9</v>
       </c>
@@ -813,7 +814,7 @@
         <v>-151.5</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" s="3">
         <v>13.8</v>
       </c>
@@ -824,7 +825,7 @@
         <v>-166.5</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" s="3">
         <v>12.8</v>
       </c>
@@ -835,7 +836,7 @@
         <v>-180.5</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" s="3">
         <v>11.6</v>
       </c>
@@ -846,7 +847,7 @@
         <v>-196.5</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" s="3">
         <v>10.5</v>
       </c>
@@ -857,7 +858,7 @@
         <v>-210.5</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" s="3">
         <v>9.5</v>
       </c>
@@ -868,7 +869,7 @@
         <v>-225.5</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" s="3">
         <v>8.1</v>
       </c>
@@ -879,7 +880,7 @@
         <v>-241.5</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" s="3">
         <v>6.9</v>
       </c>
@@ -890,7 +891,7 @@
         <v>-255.5</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20" s="3">
         <v>5.7</v>
       </c>
@@ -901,7 +902,7 @@
         <v>-271.5</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" s="3">
         <v>5</v>
       </c>
@@ -912,7 +913,7 @@
         <v>-281.5</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22" s="3">
         <v>4.4000000000000004</v>
       </c>
@@ -923,7 +924,7 @@
         <v>-288.5</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A23" s="3">
         <v>3.5</v>
       </c>
@@ -934,7 +935,7 @@
         <v>-301.5</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A24" s="3">
         <v>2.2000000000000002</v>
       </c>
@@ -945,7 +946,7 @@
         <v>-315.5</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A25" s="3">
         <v>0.2</v>
       </c>
@@ -964,12 +965,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F5976B9C-6F64-464C-90E5-C31C4813784A}">
   <dimension ref="A1:H25"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -990,7 +991,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" s="3">
         <v>27.4</v>
       </c>
@@ -1011,7 +1012,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="3">
         <v>26.2</v>
       </c>
@@ -1023,7 +1024,7 @@
       </c>
       <c r="D3" s="2"/>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" s="3">
         <v>25.1</v>
       </c>
@@ -1035,7 +1036,7 @@
       </c>
       <c r="D4" s="2"/>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5" s="3">
         <v>24.2</v>
       </c>
@@ -1046,14 +1047,14 @@
         <v>-47.5</v>
       </c>
       <c r="D5" s="2"/>
-      <c r="E5" s="7" t="s">
+      <c r="E5" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="F5" s="7"/>
-      <c r="G5" s="7"/>
-      <c r="H5" s="7"/>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="F5" s="10"/>
+      <c r="G5" s="10"/>
+      <c r="H5" s="10"/>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="3">
         <v>23.1</v>
       </c>
@@ -1064,12 +1065,12 @@
         <v>-62.5</v>
       </c>
       <c r="D6" s="2"/>
-      <c r="E6" s="7"/>
-      <c r="F6" s="7"/>
-      <c r="G6" s="7"/>
-      <c r="H6" s="7"/>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="E6" s="10"/>
+      <c r="F6" s="10"/>
+      <c r="G6" s="10"/>
+      <c r="H6" s="10"/>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="3">
         <v>21.7</v>
       </c>
@@ -1080,12 +1081,12 @@
         <v>-78.5</v>
       </c>
       <c r="D7" s="2"/>
-      <c r="E7" s="7"/>
-      <c r="F7" s="7"/>
-      <c r="G7" s="7"/>
-      <c r="H7" s="7"/>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="E7" s="10"/>
+      <c r="F7" s="10"/>
+      <c r="G7" s="10"/>
+      <c r="H7" s="10"/>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" s="3">
         <v>20.6</v>
       </c>
@@ -1096,12 +1097,12 @@
         <v>-94.5</v>
       </c>
       <c r="D8" s="2"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7"/>
-      <c r="G8" s="7"/>
-      <c r="H8" s="7"/>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="E8" s="10"/>
+      <c r="F8" s="10"/>
+      <c r="G8" s="10"/>
+      <c r="H8" s="10"/>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="3">
         <v>19.5</v>
       </c>
@@ -1112,12 +1113,12 @@
         <v>-107.5</v>
       </c>
       <c r="D9" s="2"/>
-      <c r="E9" s="7"/>
-      <c r="F9" s="7"/>
-      <c r="G9" s="7"/>
-      <c r="H9" s="7"/>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="E9" s="10"/>
+      <c r="F9" s="10"/>
+      <c r="G9" s="10"/>
+      <c r="H9" s="10"/>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A10" s="3">
         <v>18.2</v>
       </c>
@@ -1128,12 +1129,12 @@
         <v>-123.5</v>
       </c>
       <c r="D10" s="2"/>
-      <c r="E10" s="7"/>
-      <c r="F10" s="7"/>
-      <c r="G10" s="7"/>
-      <c r="H10" s="7"/>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="E10" s="10"/>
+      <c r="F10" s="10"/>
+      <c r="G10" s="10"/>
+      <c r="H10" s="10"/>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A11" s="3">
         <v>17.100000000000001</v>
       </c>
@@ -1144,12 +1145,12 @@
         <v>-137.5</v>
       </c>
       <c r="D11" s="2"/>
-      <c r="E11" s="7"/>
-      <c r="F11" s="7"/>
-      <c r="G11" s="7"/>
-      <c r="H11" s="7"/>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="E11" s="10"/>
+      <c r="F11" s="10"/>
+      <c r="G11" s="10"/>
+      <c r="H11" s="10"/>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A12" s="3">
         <v>15.9</v>
       </c>
@@ -1159,12 +1160,12 @@
       <c r="C12" s="4">
         <v>-153.5</v>
       </c>
-      <c r="E12" s="7"/>
-      <c r="F12" s="7"/>
-      <c r="G12" s="7"/>
-      <c r="H12" s="7"/>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="E12" s="10"/>
+      <c r="F12" s="10"/>
+      <c r="G12" s="10"/>
+      <c r="H12" s="10"/>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" s="3">
         <v>14.8</v>
       </c>
@@ -1174,12 +1175,12 @@
       <c r="C13" s="4">
         <v>-168.5</v>
       </c>
-      <c r="E13" s="7"/>
-      <c r="F13" s="7"/>
-      <c r="G13" s="7"/>
-      <c r="H13" s="7"/>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="E13" s="10"/>
+      <c r="F13" s="10"/>
+      <c r="G13" s="10"/>
+      <c r="H13" s="10"/>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14" s="3">
         <v>13.8</v>
       </c>
@@ -1190,7 +1191,7 @@
         <v>-182.5</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15" s="3">
         <v>12.6</v>
       </c>
@@ -1201,7 +1202,7 @@
         <v>-198.5</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A16" s="3">
         <v>11.5</v>
       </c>
@@ -1212,7 +1213,7 @@
         <v>-212.5</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" s="3">
         <v>10.5</v>
       </c>
@@ -1223,7 +1224,7 @@
         <v>-227.5</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" s="3">
         <v>9.1</v>
       </c>
@@ -1234,7 +1235,7 @@
         <v>-243.5</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" s="3">
         <v>7.9</v>
       </c>
@@ -1245,7 +1246,7 @@
         <v>-257.5</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20" s="3">
         <v>6.7</v>
       </c>
@@ -1256,7 +1257,7 @@
         <v>-273.5</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" s="3">
         <v>6</v>
       </c>
@@ -1267,7 +1268,7 @@
         <v>-283.5</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22" s="3">
         <v>5.4</v>
       </c>
@@ -1278,7 +1279,7 @@
         <v>-290.5</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A23" s="3">
         <v>4.5</v>
       </c>
@@ -1289,7 +1290,7 @@
         <v>-303.5</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A24" s="3">
         <v>3.2</v>
       </c>
@@ -1300,7 +1301,7 @@
         <v>-317.5</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A25" s="3">
         <v>0.7</v>
       </c>
@@ -1322,9 +1323,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AAFB7ADC-7EAA-424E-B0D3-74FE3B74C887}">
   <dimension ref="A1:B17"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>8</v>
       </c>
@@ -1332,7 +1333,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" s="4">
         <v>5695</v>
       </c>
@@ -1340,7 +1341,7 @@
         <v>5.8</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" s="4">
         <v>4315.6000000000004</v>
       </c>
@@ -1348,7 +1349,7 @@
         <v>11.4</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" s="4">
         <v>3316</v>
       </c>
@@ -1356,7 +1357,7 @@
         <v>16.899999999999999</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" s="4">
         <v>2777</v>
       </c>
@@ -1364,7 +1365,7 @@
         <v>20.8</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" s="4">
         <v>2143</v>
       </c>
@@ -1372,7 +1373,7 @@
         <v>26.6</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" s="4">
         <v>1735.5</v>
       </c>
@@ -1380,7 +1381,7 @@
         <v>31.5</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" s="4">
         <v>1412.5</v>
       </c>
@@ -1388,7 +1389,7 @@
         <v>36.700000000000003</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" s="4">
         <v>1171.3</v>
       </c>
@@ -1396,7 +1397,7 @@
         <v>41.2</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" s="4">
         <v>979</v>
       </c>
@@ -1404,7 +1405,7 @@
         <v>45.9</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11" s="3">
         <v>801.2</v>
       </c>
@@ -1412,7 +1413,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12" s="3">
         <v>651.79999999999995</v>
       </c>
@@ -1420,7 +1421,7 @@
         <v>56.5</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" s="3">
         <v>555.4</v>
       </c>
@@ -1428,7 +1429,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14" s="3">
         <v>478</v>
       </c>
@@ -1436,7 +1437,7 @@
         <v>65.2</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A15" s="3">
         <v>383.1</v>
       </c>
@@ -1444,7 +1445,7 @@
         <v>70.900000000000006</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A16" s="3">
         <v>330.8</v>
       </c>
@@ -1452,7 +1453,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17" s="3">
         <v>275.5</v>
       </c>
@@ -1468,67 +1469,67 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14879484-62BB-467D-9B94-6FD341A75F6E}">
   <dimension ref="A1:J17"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>8</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="E1" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="F1" s="7"/>
-      <c r="G1" s="7"/>
-      <c r="H1" s="7"/>
-      <c r="I1" s="7"/>
-      <c r="J1" s="7"/>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="F1" s="10"/>
+      <c r="G1" s="10"/>
+      <c r="H1" s="10"/>
+      <c r="I1" s="10"/>
+      <c r="J1" s="10"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" s="4">
         <v>5675</v>
       </c>
       <c r="B2" s="3">
         <v>3.8</v>
       </c>
-      <c r="E2" s="7"/>
-      <c r="F2" s="7"/>
-      <c r="G2" s="7"/>
-      <c r="H2" s="7"/>
-      <c r="I2" s="7"/>
-      <c r="J2" s="7"/>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="E2" s="10"/>
+      <c r="F2" s="10"/>
+      <c r="G2" s="10"/>
+      <c r="H2" s="10"/>
+      <c r="I2" s="10"/>
+      <c r="J2" s="10"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" s="4">
         <v>4295.6000000000004</v>
       </c>
       <c r="B3" s="3">
         <v>9.4</v>
       </c>
-      <c r="E3" s="7"/>
-      <c r="F3" s="7"/>
-      <c r="G3" s="7"/>
-      <c r="H3" s="7"/>
-      <c r="I3" s="7"/>
-      <c r="J3" s="7"/>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="E3" s="10"/>
+      <c r="F3" s="10"/>
+      <c r="G3" s="10"/>
+      <c r="H3" s="10"/>
+      <c r="I3" s="10"/>
+      <c r="J3" s="10"/>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" s="4">
         <v>3296</v>
       </c>
       <c r="B4" s="3">
         <v>14.899999999999999</v>
       </c>
-      <c r="E4" s="7"/>
-      <c r="F4" s="7"/>
-      <c r="G4" s="7"/>
-      <c r="H4" s="7"/>
-      <c r="I4" s="7"/>
-      <c r="J4" s="7"/>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="E4" s="10"/>
+      <c r="F4" s="10"/>
+      <c r="G4" s="10"/>
+      <c r="H4" s="10"/>
+      <c r="I4" s="10"/>
+      <c r="J4" s="10"/>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" s="4">
         <v>2757</v>
       </c>
@@ -1536,7 +1537,7 @@
         <v>18.8</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A6" s="4">
         <v>2123</v>
       </c>
@@ -1544,7 +1545,7 @@
         <v>24.6</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7" s="4">
         <v>1715.5</v>
       </c>
@@ -1552,7 +1553,7 @@
         <v>29.5</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" s="4">
         <v>1392.5</v>
       </c>
@@ -1560,7 +1561,7 @@
         <v>34.700000000000003</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A9" s="4">
         <v>1151.3</v>
       </c>
@@ -1568,7 +1569,7 @@
         <v>39.200000000000003</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A10" s="4">
         <v>959</v>
       </c>
@@ -1576,7 +1577,7 @@
         <v>43.9</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A11" s="3">
         <v>781.2</v>
       </c>
@@ -1584,7 +1585,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A12" s="3">
         <v>631.79999999999995</v>
       </c>
@@ -1592,7 +1593,7 @@
         <v>54.5</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A13" s="3">
         <v>535.4</v>
       </c>
@@ -1600,7 +1601,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A14" s="3">
         <v>458</v>
       </c>
@@ -1608,7 +1609,7 @@
         <v>63.2</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A15" s="3">
         <v>363.1</v>
       </c>
@@ -1616,7 +1617,7 @@
         <v>68.900000000000006</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A16" s="3">
         <v>310.8</v>
       </c>
@@ -1624,7 +1625,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17" s="3">
         <v>255.5</v>
       </c>
@@ -1643,82 +1644,82 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68FF4CBB-C579-499E-886E-8E638C13B040}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:3" ht="17.25" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>11</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="C1" s="7" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" s="3">
         <v>24.4</v>
       </c>
-      <c r="B2" s="9">
+      <c r="B2" s="8">
         <v>7.2600000000000003E-5</v>
       </c>
-      <c r="C2" s="10">
+      <c r="C2" s="9">
         <v>3.0000000000000001E-5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" s="3">
         <v>30</v>
       </c>
-      <c r="B3" s="9">
+      <c r="B3" s="8">
         <v>1.3899999999999999E-4</v>
       </c>
-      <c r="C3" s="10">
+      <c r="C3" s="9">
         <v>4.6E-5</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" s="3">
         <v>34.700000000000003</v>
       </c>
-      <c r="B4" s="9">
+      <c r="B4" s="8">
         <v>3.5300000000000002E-4</v>
       </c>
-      <c r="C4" s="10">
+      <c r="C4" s="9">
         <v>6.7000000000000002E-5</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" s="3">
         <v>40.200000000000003</v>
       </c>
-      <c r="B5" s="9">
+      <c r="B5" s="8">
         <v>7.1699999999999997E-4</v>
       </c>
-      <c r="C5" s="10">
+      <c r="C5" s="9">
         <v>1.15E-4</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" s="3">
         <v>45.1</v>
       </c>
-      <c r="B6" s="9">
+      <c r="B6" s="8">
         <v>1.6000000000000001E-3</v>
       </c>
-      <c r="C6" s="10">
+      <c r="C6" s="9">
         <v>1.7200000000000001E-4</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" s="3">
         <v>50.3</v>
       </c>
-      <c r="B7" s="9">
+      <c r="B7" s="8">
         <v>3.3400000000000001E-3</v>
       </c>
-      <c r="C7" s="10">
+      <c r="C7" s="9">
         <v>1.4999999999999999E-4</v>
       </c>
     </row>
@@ -1730,104 +1731,104 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26419247-9B67-4EF3-AD56-7F205D07E3BA}">
   <dimension ref="A1:H7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:8" ht="17.25" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>11</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="C1" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="E1" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F1" s="7"/>
-      <c r="G1" s="7"/>
-      <c r="H1" s="7"/>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="F1" s="10"/>
+      <c r="G1" s="10"/>
+      <c r="H1" s="10"/>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" s="3">
         <v>26.9</v>
       </c>
-      <c r="B2" s="9">
+      <c r="B2" s="8">
         <v>8.8599999999999999E-5</v>
       </c>
-      <c r="C2" s="10">
+      <c r="C2" s="9">
         <v>9.0000000000000006E-5</v>
       </c>
-      <c r="E2" s="7"/>
-      <c r="F2" s="7"/>
-      <c r="G2" s="7"/>
-      <c r="H2" s="7"/>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="E2" s="10"/>
+      <c r="F2" s="10"/>
+      <c r="G2" s="10"/>
+      <c r="H2" s="10"/>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="3">
         <v>32.5</v>
       </c>
-      <c r="B3" s="9">
+      <c r="B3" s="8">
         <v>1.55E-4</v>
       </c>
-      <c r="C3" s="10">
+      <c r="C3" s="9">
         <v>1.06E-4</v>
       </c>
-      <c r="E3" s="7"/>
-      <c r="F3" s="7"/>
-      <c r="G3" s="7"/>
-      <c r="H3" s="7"/>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="E3" s="10"/>
+      <c r="F3" s="10"/>
+      <c r="G3" s="10"/>
+      <c r="H3" s="10"/>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" s="3">
         <v>37.200000000000003</v>
       </c>
-      <c r="B4" s="9">
+      <c r="B4" s="8">
         <v>3.6900000000000002E-4</v>
       </c>
-      <c r="C4" s="10">
+      <c r="C4" s="9">
         <v>1.27E-4</v>
       </c>
-      <c r="E4" s="7"/>
-      <c r="F4" s="7"/>
-      <c r="G4" s="7"/>
-      <c r="H4" s="7"/>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="E4" s="10"/>
+      <c r="F4" s="10"/>
+      <c r="G4" s="10"/>
+      <c r="H4" s="10"/>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5" s="3">
         <v>42.7</v>
       </c>
-      <c r="B5" s="9">
+      <c r="B5" s="8">
         <v>7.3299999999999993E-4</v>
       </c>
-      <c r="C5" s="10">
+      <c r="C5" s="9">
         <v>1.75E-4</v>
       </c>
-      <c r="E5" s="7"/>
-      <c r="F5" s="7"/>
-      <c r="G5" s="7"/>
-      <c r="H5" s="7"/>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="E5" s="10"/>
+      <c r="F5" s="10"/>
+      <c r="G5" s="10"/>
+      <c r="H5" s="10"/>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="3">
         <v>47.6</v>
       </c>
-      <c r="B6" s="9">
+      <c r="B6" s="8">
         <v>1.616E-3</v>
       </c>
-      <c r="C6" s="10">
+      <c r="C6" s="9">
         <v>2.32E-4</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="3">
         <v>52.8</v>
       </c>
-      <c r="B7" s="9">
+      <c r="B7" s="8">
         <v>3.356E-3</v>
       </c>
-      <c r="C7" s="10">
+      <c r="C7" s="9">
         <v>2.0999999999999998E-4</v>
       </c>
     </row>
@@ -1837,4 +1838,13 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E9A0E81F-3D86-D54E-B3A3-87437B7BE8EF}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>